<commit_message>
MD80 files fit for trade studies
</commit_message>
<xml_diff>
--- a/William MD80 Files/DesconLampe4138.xlsx
+++ b/William MD80 Files/DesconLampe4138.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamlampe/Documents/GitHub/ASEN4138_AircraftDesign/William MD80 Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF13E12A-C3A3-0645-9F6D-7AEC6160956B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CB1779-D05B-ED42-ABC2-A0815DDC9699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="1" activeTab="1" xr2:uid="{904FC4B5-3CDE-421B-8E98-23A2C72E8C1E}"/>
   </bookViews>
@@ -360,7 +360,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="243">
   <si>
     <t>Length_f</t>
   </si>
@@ -1070,32 +1070,32 @@
     <t>Prop_Dia</t>
   </si>
   <si>
-    <t>all stats -&gt; after are for per engine</t>
-  </si>
-  <si>
-    <t>Prop -&gt; jet = 0</t>
-  </si>
-  <si>
-    <t>Turbocharge is from sea level to 8,000 ft</t>
-  </si>
-  <si>
-    <t>Electric -&gt; jet = 0</t>
-  </si>
-  <si>
-    <t>MD80</t>
-  </si>
-  <si>
     <t>DSMA-523A</t>
   </si>
   <si>
     <t>NACA 0004</t>
+  </si>
+  <si>
+    <t>MD80_1</t>
+  </si>
+  <si>
+    <t>MD80_2</t>
+  </si>
+  <si>
+    <t>MD80_3</t>
+  </si>
+  <si>
+    <t>MD80_4</t>
+  </si>
+  <si>
+    <t>MD80_5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1142,6 +1142,13 @@
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="14">
@@ -1224,7 +1231,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1247,11 +1254,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1319,7 +1339,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3335,7 +3360,7 @@
     </row>
     <row r="2" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>210</v>
@@ -3488,8 +3513,620 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="F3" s="4">
+        <v>147.67060000000001</v>
+      </c>
+      <c r="G3" s="4">
+        <v>15</v>
+      </c>
+      <c r="H3" s="4">
+        <f>F3/G3</f>
+        <v>9.8447066666666672</v>
+      </c>
+      <c r="I3" s="4">
+        <f>0.25*PI()*(G3)^2</f>
+        <v>176.71458676442586</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
+        <f>PI()*G3*F3</f>
+        <v>6958.8130816679532</v>
+      </c>
+      <c r="L3" s="4">
+        <v>1</v>
+      </c>
+      <c r="M3" s="4">
+        <v>2</v>
+      </c>
+      <c r="N3" s="4">
+        <v>1209</v>
+      </c>
+      <c r="O3" s="4">
+        <v>2500</v>
+      </c>
+      <c r="P3" s="4">
+        <f>(107.67717^2)/N3</f>
+        <v>9.5900520588990084</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="R3" s="4">
+        <v>35</v>
+      </c>
+      <c r="S3" s="4">
+        <v>30</v>
+      </c>
+      <c r="T3" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U3" s="4">
+        <f>0.25*N3</f>
+        <v>302.25</v>
+      </c>
+      <c r="V3" s="4">
+        <f>2*U3</f>
+        <v>604.5</v>
+      </c>
+      <c r="W3" s="4">
+        <f>((107.67717/3)^2)/U3</f>
+        <v>4.2622453595106693</v>
+      </c>
+      <c r="X3" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="Y3" s="4">
+        <f>35</f>
+        <v>35</v>
+      </c>
+      <c r="Z3" s="4">
+        <f>(15+(15*0.4))/2</f>
+        <v>10.5</v>
+      </c>
+      <c r="AA3" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="4">
+        <v>302.25</v>
+      </c>
+      <c r="AJ3" s="4">
+        <v>604.5</v>
+      </c>
+      <c r="AK3" s="4">
+        <v>4.2622450000000001</v>
+      </c>
+      <c r="AL3" s="4">
+        <v>1</v>
+      </c>
+      <c r="AM3" s="4">
+        <v>35</v>
+      </c>
+      <c r="AN3" s="4">
+        <v>10.5</v>
+      </c>
+      <c r="AO3" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AQ3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AR3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AS3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AT3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AU3" s="4">
+        <v>0</v>
+      </c>
+      <c r="AV3" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="F4" s="4">
+        <v>147.67060000000001</v>
+      </c>
+      <c r="G4" s="4">
+        <v>15</v>
+      </c>
+      <c r="H4" s="4">
+        <f>F4/G4</f>
+        <v>9.8447066666666672</v>
+      </c>
+      <c r="I4" s="4">
+        <f>0.25*PI()*(G4)^2</f>
+        <v>176.71458676442586</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <f>PI()*G4*F4</f>
+        <v>6958.8130816679532</v>
+      </c>
+      <c r="L4" s="4">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4">
+        <v>2</v>
+      </c>
+      <c r="N4" s="4">
+        <v>1209</v>
+      </c>
+      <c r="O4" s="4">
+        <v>2500</v>
+      </c>
+      <c r="P4" s="4">
+        <f>(107.67717^2)/N4</f>
+        <v>9.5900520588990084</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="R4" s="4">
+        <v>35</v>
+      </c>
+      <c r="S4" s="4">
+        <v>30</v>
+      </c>
+      <c r="T4" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U4" s="4">
+        <f>0.25*N4</f>
+        <v>302.25</v>
+      </c>
+      <c r="V4" s="4">
+        <f>2*U4</f>
+        <v>604.5</v>
+      </c>
+      <c r="W4" s="4">
+        <f>((107.67717/3)^2)/U4</f>
+        <v>4.2622453595106693</v>
+      </c>
+      <c r="X4" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="Y4" s="4">
+        <f>35</f>
+        <v>35</v>
+      </c>
+      <c r="Z4" s="4">
+        <f>(15+(15*0.4))/2</f>
+        <v>10.5</v>
+      </c>
+      <c r="AA4" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="4">
+        <v>302.25</v>
+      </c>
+      <c r="AJ4" s="4">
+        <v>604.5</v>
+      </c>
+      <c r="AK4" s="4">
+        <v>4.2622450000000001</v>
+      </c>
+      <c r="AL4" s="4">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="4">
+        <v>35</v>
+      </c>
+      <c r="AN4" s="4">
+        <v>10.5</v>
+      </c>
+      <c r="AO4" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AR4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AS4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AT4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AU4" s="4">
+        <v>0</v>
+      </c>
+      <c r="AV4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="F5" s="4">
+        <v>147.67060000000001</v>
+      </c>
+      <c r="G5" s="4">
+        <v>15</v>
+      </c>
+      <c r="H5" s="4">
+        <f>F5/G5</f>
+        <v>9.8447066666666672</v>
+      </c>
+      <c r="I5" s="4">
+        <f>0.25*PI()*(G5)^2</f>
+        <v>176.71458676442586</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
+        <f>PI()*G5*F5</f>
+        <v>6958.8130816679532</v>
+      </c>
+      <c r="L5" s="4">
+        <v>1</v>
+      </c>
+      <c r="M5" s="4">
+        <v>2</v>
+      </c>
+      <c r="N5" s="4">
+        <v>1209</v>
+      </c>
+      <c r="O5" s="4">
+        <v>2500</v>
+      </c>
+      <c r="P5" s="4">
+        <f>(107.67717^2)/N5</f>
+        <v>9.5900520588990084</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="R5" s="4">
+        <v>35</v>
+      </c>
+      <c r="S5" s="4">
+        <v>30</v>
+      </c>
+      <c r="T5" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U5" s="4">
+        <f>0.25*N5</f>
+        <v>302.25</v>
+      </c>
+      <c r="V5" s="4">
+        <f>2*U5</f>
+        <v>604.5</v>
+      </c>
+      <c r="W5" s="4">
+        <f>((107.67717/3)^2)/U5</f>
+        <v>4.2622453595106693</v>
+      </c>
+      <c r="X5" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="Y5" s="4">
+        <f>35</f>
+        <v>35</v>
+      </c>
+      <c r="Z5" s="4">
+        <f>(15+(15*0.4))/2</f>
+        <v>10.5</v>
+      </c>
+      <c r="AA5" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="4">
+        <v>302.25</v>
+      </c>
+      <c r="AJ5" s="4">
+        <v>604.5</v>
+      </c>
+      <c r="AK5" s="4">
+        <v>4.2622450000000001</v>
+      </c>
+      <c r="AL5" s="4">
+        <v>1</v>
+      </c>
+      <c r="AM5" s="4">
+        <v>35</v>
+      </c>
+      <c r="AN5" s="4">
+        <v>10.5</v>
+      </c>
+      <c r="AO5" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AQ5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AR5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AS5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AT5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AU5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AV5" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A6" s="29" t="s">
+        <v>242</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="C6" s="30">
+        <v>0</v>
+      </c>
+      <c r="D6" s="30">
+        <v>0.76</v>
+      </c>
+      <c r="E6" s="30">
+        <v>0.76</v>
+      </c>
+      <c r="F6" s="30">
+        <v>147.67060000000001</v>
+      </c>
+      <c r="G6" s="30">
+        <v>15</v>
+      </c>
+      <c r="H6" s="30">
+        <v>9.8447069999999997</v>
+      </c>
+      <c r="I6" s="30">
+        <v>176.71459999999999</v>
+      </c>
+      <c r="J6" s="30">
+        <v>0</v>
+      </c>
+      <c r="K6" s="30">
+        <v>6958.8130000000001</v>
+      </c>
+      <c r="L6" s="30">
+        <v>1</v>
+      </c>
+      <c r="M6" s="30">
+        <v>2</v>
+      </c>
+      <c r="N6" s="30">
+        <v>1209</v>
+      </c>
+      <c r="O6" s="30">
+        <v>2500</v>
+      </c>
+      <c r="P6" s="30">
+        <v>9.590052</v>
+      </c>
+      <c r="Q6" s="30">
+        <v>0.25</v>
+      </c>
+      <c r="R6" s="30">
+        <v>35</v>
+      </c>
+      <c r="S6" s="30">
+        <v>30</v>
+      </c>
+      <c r="T6" s="30">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U6" s="30">
+        <v>302.25</v>
+      </c>
+      <c r="V6" s="30">
+        <v>604.5</v>
+      </c>
+      <c r="W6" s="30">
+        <v>4.2622450000000001</v>
+      </c>
+      <c r="X6" s="30">
+        <v>0.4</v>
+      </c>
+      <c r="Y6" s="30">
+        <v>35</v>
+      </c>
+      <c r="Z6" s="30">
+        <v>10.5</v>
+      </c>
+      <c r="AA6" s="30">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="30">
+        <v>302.25</v>
+      </c>
+      <c r="AJ6" s="30">
+        <v>604.5</v>
+      </c>
+      <c r="AK6" s="30">
+        <v>4.2622450000000001</v>
+      </c>
+      <c r="AL6" s="30">
+        <v>1</v>
+      </c>
+      <c r="AM6" s="30">
+        <v>35</v>
+      </c>
+      <c r="AN6" s="30">
+        <v>10.5</v>
+      </c>
+      <c r="AO6" s="30">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AR6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AS6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AT6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AU6" s="30">
+        <v>0</v>
+      </c>
+      <c r="AV6" s="30">
+        <v>0</v>
+      </c>
+    </row>
     <row r="16" spans="1:48" s="21" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -3498,7 +4135,7 @@
           <x14:formula1>
             <xm:f>Lists!$B$2:$B$19</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B15</xm:sqref>
+          <xm:sqref>B7:B15</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3692,10 +4329,10 @@
     </row>
     <row r="2" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="C2" s="10">
         <v>0.11</v>
@@ -3819,7 +4456,7 @@
         <v>6.3699999999999998E-3</v>
       </c>
       <c r="AQ2" s="10" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="AR2" s="10">
         <v>0.04</v>
@@ -3856,34 +4493,664 @@
       </c>
     </row>
     <row r="3" spans="1:54" x14ac:dyDescent="0.2">
-      <c r="J3"/>
-      <c r="K3"/>
-      <c r="L3"/>
-      <c r="M3"/>
-      <c r="N3"/>
-      <c r="O3"/>
-      <c r="P3"/>
-      <c r="Q3"/>
-      <c r="S3"/>
-      <c r="T3"/>
-      <c r="V3"/>
-      <c r="X3"/>
-      <c r="Y3"/>
-      <c r="Z3"/>
-      <c r="AA3"/>
-      <c r="AB3"/>
-      <c r="AC3"/>
-      <c r="AD3"/>
-      <c r="AE3"/>
-      <c r="AF3"/>
-      <c r="AG3"/>
-      <c r="AH3"/>
-      <c r="AI3"/>
-      <c r="AJ3"/>
-      <c r="AL3"/>
-      <c r="AM3"/>
-      <c r="AN3"/>
-      <c r="AO3"/>
+      <c r="A3" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C3" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="D3" s="10">
+        <v>0.36</v>
+      </c>
+      <c r="E3" s="10">
+        <v>-0.36480000000000001</v>
+      </c>
+      <c r="F3" s="10">
+        <v>-0.22969999999999999</v>
+      </c>
+      <c r="G3" s="10">
+        <v>-9.06E-2</v>
+      </c>
+      <c r="H3" s="10">
+        <v>9.1499999999999998E-2</v>
+      </c>
+      <c r="I3" s="10">
+        <v>0.25209999999999999</v>
+      </c>
+      <c r="J3" s="10">
+        <v>0.3926</v>
+      </c>
+      <c r="K3" s="10">
+        <v>0.4924</v>
+      </c>
+      <c r="L3" s="10">
+        <v>0.59919999999999995</v>
+      </c>
+      <c r="M3" s="10">
+        <v>0.70809999999999995</v>
+      </c>
+      <c r="N3" s="10">
+        <v>0.81489999999999996</v>
+      </c>
+      <c r="O3" s="10">
+        <v>0.92130000000000001</v>
+      </c>
+      <c r="P3" s="10">
+        <v>1.0299</v>
+      </c>
+      <c r="Q3" s="10">
+        <v>1.1337999999999999</v>
+      </c>
+      <c r="R3" s="10">
+        <v>1.2350000000000001</v>
+      </c>
+      <c r="S3" s="10">
+        <v>1.3317000000000001</v>
+      </c>
+      <c r="T3" s="10">
+        <v>1.4271</v>
+      </c>
+      <c r="U3" s="10">
+        <v>1.5059</v>
+      </c>
+      <c r="V3" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="W3" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="X3" s="10">
+        <v>1.2370000000000001E-2</v>
+      </c>
+      <c r="Y3" s="10">
+        <v>1.1509999999999999E-2</v>
+      </c>
+      <c r="Z3" s="10">
+        <v>1.082E-2</v>
+      </c>
+      <c r="AA3" s="10">
+        <v>9.1400000000000006E-3</v>
+      </c>
+      <c r="AB3" s="10">
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AC3" s="10">
+        <v>8.1300000000000001E-3</v>
+      </c>
+      <c r="AD3" s="10">
+        <v>1.027E-2</v>
+      </c>
+      <c r="AE3" s="10">
+        <v>1.1220000000000001E-2</v>
+      </c>
+      <c r="AF3" s="10">
+        <v>1.2160000000000001E-2</v>
+      </c>
+      <c r="AG3" s="10">
+        <v>1.312E-2</v>
+      </c>
+      <c r="AH3" s="10">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="AI3" s="10">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="AJ3" s="10">
+        <v>1.651E-2</v>
+      </c>
+      <c r="AK3" s="10">
+        <v>1.806E-2</v>
+      </c>
+      <c r="AL3" s="10">
+        <v>1.9970000000000002E-2</v>
+      </c>
+      <c r="AM3" s="10">
+        <v>2.1649999999999999E-2</v>
+      </c>
+      <c r="AN3" s="10">
+        <v>2.487E-2</v>
+      </c>
+      <c r="AO3" s="10">
+        <v>2.726E-2</v>
+      </c>
+      <c r="AP3" s="10">
+        <f>MIN(X3:AO3)</f>
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AQ3" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="AR3" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AS3" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AT3" s="10">
+        <v>0</v>
+      </c>
+      <c r="AU3" s="10">
+        <v>0</v>
+      </c>
+      <c r="AV3" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW3" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="AX3" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AY3" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AZ3" s="10">
+        <v>0</v>
+      </c>
+      <c r="BA3" s="10">
+        <v>0</v>
+      </c>
+      <c r="BB3" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="D4" s="10">
+        <v>0.36</v>
+      </c>
+      <c r="E4" s="10">
+        <v>-0.36480000000000001</v>
+      </c>
+      <c r="F4" s="10">
+        <v>-0.22969999999999999</v>
+      </c>
+      <c r="G4" s="10">
+        <v>-9.06E-2</v>
+      </c>
+      <c r="H4" s="10">
+        <v>9.1499999999999998E-2</v>
+      </c>
+      <c r="I4" s="10">
+        <v>0.25209999999999999</v>
+      </c>
+      <c r="J4" s="10">
+        <v>0.3926</v>
+      </c>
+      <c r="K4" s="10">
+        <v>0.4924</v>
+      </c>
+      <c r="L4" s="10">
+        <v>0.59919999999999995</v>
+      </c>
+      <c r="M4" s="10">
+        <v>0.70809999999999995</v>
+      </c>
+      <c r="N4" s="10">
+        <v>0.81489999999999996</v>
+      </c>
+      <c r="O4" s="10">
+        <v>0.92130000000000001</v>
+      </c>
+      <c r="P4" s="10">
+        <v>1.0299</v>
+      </c>
+      <c r="Q4" s="10">
+        <v>1.1337999999999999</v>
+      </c>
+      <c r="R4" s="10">
+        <v>1.2350000000000001</v>
+      </c>
+      <c r="S4" s="10">
+        <v>1.3317000000000001</v>
+      </c>
+      <c r="T4" s="10">
+        <v>1.4271</v>
+      </c>
+      <c r="U4" s="10">
+        <v>1.5059</v>
+      </c>
+      <c r="V4" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="W4" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="X4" s="10">
+        <v>1.2370000000000001E-2</v>
+      </c>
+      <c r="Y4" s="10">
+        <v>1.1509999999999999E-2</v>
+      </c>
+      <c r="Z4" s="10">
+        <v>1.082E-2</v>
+      </c>
+      <c r="AA4" s="10">
+        <v>9.1400000000000006E-3</v>
+      </c>
+      <c r="AB4" s="10">
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AC4" s="10">
+        <v>8.1300000000000001E-3</v>
+      </c>
+      <c r="AD4" s="10">
+        <v>1.027E-2</v>
+      </c>
+      <c r="AE4" s="10">
+        <v>1.1220000000000001E-2</v>
+      </c>
+      <c r="AF4" s="10">
+        <v>1.2160000000000001E-2</v>
+      </c>
+      <c r="AG4" s="10">
+        <v>1.312E-2</v>
+      </c>
+      <c r="AH4" s="10">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="AI4" s="10">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="AJ4" s="10">
+        <v>1.651E-2</v>
+      </c>
+      <c r="AK4" s="10">
+        <v>1.806E-2</v>
+      </c>
+      <c r="AL4" s="10">
+        <v>1.9970000000000002E-2</v>
+      </c>
+      <c r="AM4" s="10">
+        <v>2.1649999999999999E-2</v>
+      </c>
+      <c r="AN4" s="10">
+        <v>2.487E-2</v>
+      </c>
+      <c r="AO4" s="10">
+        <v>2.726E-2</v>
+      </c>
+      <c r="AP4" s="10">
+        <f>MIN(X4:AO4)</f>
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AQ4" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="AR4" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AS4" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AT4" s="10">
+        <v>0</v>
+      </c>
+      <c r="AU4" s="10">
+        <v>0</v>
+      </c>
+      <c r="AV4" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW4" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="AX4" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AY4" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AZ4" s="10">
+        <v>0</v>
+      </c>
+      <c r="BA4" s="10">
+        <v>0</v>
+      </c>
+      <c r="BB4" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="D5" s="10">
+        <v>0.36</v>
+      </c>
+      <c r="E5" s="10">
+        <v>-0.36480000000000001</v>
+      </c>
+      <c r="F5" s="10">
+        <v>-0.22969999999999999</v>
+      </c>
+      <c r="G5" s="10">
+        <v>-9.06E-2</v>
+      </c>
+      <c r="H5" s="10">
+        <v>9.1499999999999998E-2</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0.25209999999999999</v>
+      </c>
+      <c r="J5" s="10">
+        <v>0.3926</v>
+      </c>
+      <c r="K5" s="10">
+        <v>0.4924</v>
+      </c>
+      <c r="L5" s="10">
+        <v>0.59919999999999995</v>
+      </c>
+      <c r="M5" s="10">
+        <v>0.70809999999999995</v>
+      </c>
+      <c r="N5" s="10">
+        <v>0.81489999999999996</v>
+      </c>
+      <c r="O5" s="10">
+        <v>0.92130000000000001</v>
+      </c>
+      <c r="P5" s="10">
+        <v>1.0299</v>
+      </c>
+      <c r="Q5" s="10">
+        <v>1.1337999999999999</v>
+      </c>
+      <c r="R5" s="10">
+        <v>1.2350000000000001</v>
+      </c>
+      <c r="S5" s="10">
+        <v>1.3317000000000001</v>
+      </c>
+      <c r="T5" s="10">
+        <v>1.4271</v>
+      </c>
+      <c r="U5" s="10">
+        <v>1.5059</v>
+      </c>
+      <c r="V5" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="W5" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="X5" s="10">
+        <v>1.2370000000000001E-2</v>
+      </c>
+      <c r="Y5" s="10">
+        <v>1.1509999999999999E-2</v>
+      </c>
+      <c r="Z5" s="10">
+        <v>1.082E-2</v>
+      </c>
+      <c r="AA5" s="10">
+        <v>9.1400000000000006E-3</v>
+      </c>
+      <c r="AB5" s="10">
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AC5" s="10">
+        <v>8.1300000000000001E-3</v>
+      </c>
+      <c r="AD5" s="10">
+        <v>1.027E-2</v>
+      </c>
+      <c r="AE5" s="10">
+        <v>1.1220000000000001E-2</v>
+      </c>
+      <c r="AF5" s="10">
+        <v>1.2160000000000001E-2</v>
+      </c>
+      <c r="AG5" s="10">
+        <v>1.312E-2</v>
+      </c>
+      <c r="AH5" s="10">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="AI5" s="10">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="AJ5" s="10">
+        <v>1.651E-2</v>
+      </c>
+      <c r="AK5" s="10">
+        <v>1.806E-2</v>
+      </c>
+      <c r="AL5" s="10">
+        <v>1.9970000000000002E-2</v>
+      </c>
+      <c r="AM5" s="10">
+        <v>2.1649999999999999E-2</v>
+      </c>
+      <c r="AN5" s="10">
+        <v>2.487E-2</v>
+      </c>
+      <c r="AO5" s="10">
+        <v>2.726E-2</v>
+      </c>
+      <c r="AP5" s="10">
+        <f>MIN(X5:AO5)</f>
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AQ5" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="AR5" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AS5" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AT5" s="10">
+        <v>0</v>
+      </c>
+      <c r="AU5" s="10">
+        <v>0</v>
+      </c>
+      <c r="AV5" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW5" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="AX5" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AY5" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AZ5" s="10">
+        <v>0</v>
+      </c>
+      <c r="BA5" s="10">
+        <v>0</v>
+      </c>
+      <c r="BB5" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="D6" s="10">
+        <v>0.36</v>
+      </c>
+      <c r="E6" s="10">
+        <v>-0.36480000000000001</v>
+      </c>
+      <c r="F6" s="10">
+        <v>-0.22969999999999999</v>
+      </c>
+      <c r="G6" s="10">
+        <v>-9.06E-2</v>
+      </c>
+      <c r="H6" s="10">
+        <v>9.1499999999999998E-2</v>
+      </c>
+      <c r="I6" s="10">
+        <v>0.25209999999999999</v>
+      </c>
+      <c r="J6" s="10">
+        <v>0.3926</v>
+      </c>
+      <c r="K6" s="10">
+        <v>0.4924</v>
+      </c>
+      <c r="L6" s="10">
+        <v>0.59919999999999995</v>
+      </c>
+      <c r="M6" s="10">
+        <v>0.70809999999999995</v>
+      </c>
+      <c r="N6" s="10">
+        <v>0.81489999999999996</v>
+      </c>
+      <c r="O6" s="10">
+        <v>0.92130000000000001</v>
+      </c>
+      <c r="P6" s="10">
+        <v>1.0299</v>
+      </c>
+      <c r="Q6" s="10">
+        <v>1.1337999999999999</v>
+      </c>
+      <c r="R6" s="10">
+        <v>1.2350000000000001</v>
+      </c>
+      <c r="S6" s="10">
+        <v>1.3317000000000001</v>
+      </c>
+      <c r="T6" s="10">
+        <v>1.4271</v>
+      </c>
+      <c r="U6" s="10">
+        <v>1.5059</v>
+      </c>
+      <c r="V6" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="W6" s="10">
+        <v>1.5843</v>
+      </c>
+      <c r="X6" s="10">
+        <v>1.2370000000000001E-2</v>
+      </c>
+      <c r="Y6" s="10">
+        <v>1.1509999999999999E-2</v>
+      </c>
+      <c r="Z6" s="10">
+        <v>1.082E-2</v>
+      </c>
+      <c r="AA6" s="10">
+        <v>9.1400000000000006E-3</v>
+      </c>
+      <c r="AB6" s="10">
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AC6" s="10">
+        <v>8.1300000000000001E-3</v>
+      </c>
+      <c r="AD6" s="10">
+        <v>1.027E-2</v>
+      </c>
+      <c r="AE6" s="10">
+        <v>1.1220000000000001E-2</v>
+      </c>
+      <c r="AF6" s="10">
+        <v>1.2160000000000001E-2</v>
+      </c>
+      <c r="AG6" s="10">
+        <v>1.312E-2</v>
+      </c>
+      <c r="AH6" s="10">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="AI6" s="10">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="AJ6" s="10">
+        <v>1.651E-2</v>
+      </c>
+      <c r="AK6" s="10">
+        <v>1.806E-2</v>
+      </c>
+      <c r="AL6" s="10">
+        <v>1.9970000000000002E-2</v>
+      </c>
+      <c r="AM6" s="10">
+        <v>2.1649999999999999E-2</v>
+      </c>
+      <c r="AN6" s="10">
+        <v>2.487E-2</v>
+      </c>
+      <c r="AO6" s="10">
+        <v>2.726E-2</v>
+      </c>
+      <c r="AP6" s="10">
+        <f>MIN(X6:AO6)</f>
+        <v>6.3699999999999998E-3</v>
+      </c>
+      <c r="AQ6" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="AR6" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AS6" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AT6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AU6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AV6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW6" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="AX6" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="AY6" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="AZ6" s="10">
+        <v>0</v>
+      </c>
+      <c r="BA6" s="10">
+        <v>0</v>
+      </c>
+      <c r="BB6" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:54" s="22" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
@@ -3963,7 +5230,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B2" t="s">
         <v>185</v>
@@ -4017,27 +5284,233 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>19500</v>
+      </c>
+      <c r="E3">
+        <v>0.73</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0.2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>19500</v>
+      </c>
+      <c r="E4">
+        <v>0.73</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0.2</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>19500</v>
+      </c>
+      <c r="E5">
+        <v>0.73</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0.2</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+    </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D6" t="s">
-        <v>236</v>
-      </c>
-      <c r="H6" s="29">
+      <c r="A6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>19500</v>
+      </c>
+      <c r="E6">
+        <v>0.73</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>0.2</v>
       </c>
-      <c r="I6" t="s">
-        <v>237</v>
-      </c>
-      <c r="M6" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D7" t="s">
-        <v>238</v>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:18" s="20" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
   <extLst>
@@ -4047,7 +5520,7 @@
           <x14:formula1>
             <xm:f>Lists!$A$2:$A$7</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B15 B2</xm:sqref>
+          <xm:sqref>B2:B15</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>